<commit_message>
Fix Windows Fatal COM errors, improve pyrefly type safety, and fix VSCode pytest discovery
</commit_message>
<xml_diff>
--- a/tests/table.xlsx
+++ b/tests/table.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P61"/>
+  <dimension ref="A1:P73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4205,6 +4205,438 @@
       <c r="O61" t="inlineStr"/>
       <c r="P61" t="inlineStr"/>
     </row>
+    <row r="62">
+      <c r="A62" s="1" t="n">
+        <v>60</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>610</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr"/>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr"/>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr"/>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="inlineStr"/>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>000402</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>9130</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>0020</t>
+        </is>
+      </c>
+      <c r="O62" t="inlineStr"/>
+      <c r="P62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="1" t="n">
+        <v>61</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>620</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr"/>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr"/>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>000402</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>9130</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>0020</t>
+        </is>
+      </c>
+      <c r="O63" t="inlineStr"/>
+      <c r="P63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="1" t="n">
+        <v>62</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>630</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr"/>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr"/>
+      <c r="J64" t="inlineStr"/>
+      <c r="K64" t="inlineStr"/>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>000402</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>9130</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>0020</t>
+        </is>
+      </c>
+      <c r="O64" t="inlineStr"/>
+      <c r="P64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="1" t="n">
+        <v>63</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>640</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr"/>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr"/>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr"/>
+      <c r="J65" t="inlineStr"/>
+      <c r="K65" t="inlineStr"/>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>000402</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>9130</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>0020</t>
+        </is>
+      </c>
+      <c r="O65" t="inlineStr"/>
+      <c r="P65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="1" t="n">
+        <v>64</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>650</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr"/>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr"/>
+      <c r="J66" t="inlineStr"/>
+      <c r="K66" t="inlineStr"/>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>000402</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>9130</t>
+        </is>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>0020</t>
+        </is>
+      </c>
+      <c r="O66" t="inlineStr"/>
+      <c r="P66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="1" t="n">
+        <v>65</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>660</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr"/>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr"/>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr"/>
+      <c r="J67" t="inlineStr"/>
+      <c r="K67" t="inlineStr"/>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>000402</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>9130</t>
+        </is>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>0020</t>
+        </is>
+      </c>
+      <c r="O67" t="inlineStr"/>
+      <c r="P67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="1" t="n">
+        <v>66</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>670</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr"/>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr"/>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr"/>
+      <c r="J68" t="inlineStr"/>
+      <c r="K68" t="inlineStr"/>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>000402</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>9130</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>0020</t>
+        </is>
+      </c>
+      <c r="O68" t="inlineStr"/>
+      <c r="P68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="1" t="n">
+        <v>67</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>680</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr"/>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr"/>
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr"/>
+      <c r="J69" t="inlineStr"/>
+      <c r="K69" t="inlineStr"/>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>000402</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>9130</t>
+        </is>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>0020</t>
+        </is>
+      </c>
+      <c r="O69" t="inlineStr"/>
+      <c r="P69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="1" t="n">
+        <v>68</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>690</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr"/>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr"/>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr"/>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr"/>
+      <c r="J70" t="inlineStr"/>
+      <c r="K70" t="inlineStr"/>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>000402</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>9130</t>
+        </is>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>0020</t>
+        </is>
+      </c>
+      <c r="O70" t="inlineStr"/>
+      <c r="P70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="1" t="n">
+        <v>69</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>700</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr"/>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr"/>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr"/>
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="inlineStr"/>
+      <c r="J71" t="inlineStr"/>
+      <c r="K71" t="inlineStr"/>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>000402</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>9130</t>
+        </is>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>0020</t>
+        </is>
+      </c>
+      <c r="O71" t="inlineStr"/>
+      <c r="P71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="1" t="n">
+        <v>70</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>710</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr"/>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr"/>
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr"/>
+      <c r="J72" t="inlineStr"/>
+      <c r="K72" t="inlineStr"/>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>000402</t>
+        </is>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>9130</t>
+        </is>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>0020</t>
+        </is>
+      </c>
+      <c r="O72" t="inlineStr"/>
+      <c r="P72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="1" t="n">
+        <v>71</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>720</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr"/>
+      <c r="D73" t="inlineStr"/>
+      <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" t="inlineStr"/>
+      <c r="H73" t="inlineStr"/>
+      <c r="I73" t="inlineStr"/>
+      <c r="J73" t="inlineStr"/>
+      <c r="K73" t="inlineStr"/>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>000402</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>9130</t>
+        </is>
+      </c>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>0020</t>
+        </is>
+      </c>
+      <c r="O73" t="inlineStr"/>
+      <c r="P73" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>